<commit_message>
RC1: EB21A-02-C footprint verified against the Adam Tech drawing (rev B); J1-J4 re-placed, board re-routed
Hole 1.30 mm, body 10.6 x 8.5 mm, wire entry toward the board edge; VERIFY_MECHANICAL_DRAWING removed
for this part only. ERC 0; DRC: 0 electrical, 4 silkscreen warnings, 0 unconnected.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HV1TCrYnLTcNjmYdFqCPLo
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
+++ b/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (FOOTPRINT: VERIFY_MECHANICAL_DRAWING)</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C_PROVISIONAL</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C_PROVISIONAL</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (FOOTPRINT: VERIFY_MECHANICAL_DRAWING)</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -4098,12 +4098,12 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C_PROVISIONAL</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C_PROVISIONAL</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (FOOTPRINT: VERIFY_MECHANICAL_DRAWING)</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C_PROVISIONAL</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C_PROVISIONAL</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (FOOTPRINT: VERIFY_MECHANICAL_DRAWING)</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -4274,12 +4274,12 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C_PROVISIONAL</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C_PROVISIONAL</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">

</xml_diff>

<commit_message>
RC1: reconcile user-relayed manufacturer data (USER_RELAYED_MANUFACTURER)
- audit report MANUFACTURER_DATA_RECONCILIATION.md; INA228/STM32/IRLML0060/LMR14006Y/CP2102N/VO610A/TC74 pin maps match the relayed data
- ISO7721 pin-direction conflict left unresolved (needs the TI pin diagram); CP2102N VBUS reference connection open
- LMR14006Y: 95 ns TON_MIN analysis (15 V marginal, 24.4 V below TON_MIN); 1.5SMBJ48A vs INA228 85 V clamp-vs-current analysis
- firmware: INA228 IMAX 30 A -> 20 A (SHUNT_CAL 1250) + test
- fix: TC74 probe PCB had been left unrouted by the schematic step; re-routed, DRC 0; schematic step no longer rebuilds it

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HV1TCrYnLTcNjmYdFqCPLo
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
+++ b/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
@@ -2142,9 +2142,9 @@
           <t>Package_QFP:LQFP-64_10x10mm_P0.5mm</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -3078,9 +3078,9 @@
           <t>Package_DFN_QFN:SiliconLabs_QFN-20-1EP_3x3mm_P0.5mm_EP1.8x1.8mm</t>
         </is>
       </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -3162,9 +3162,9 @@
           <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -4370,9 +4370,9 @@
           <t>Package_TO_SOT_SMD:SOT-23</t>
         </is>
       </c>
-      <c r="J47" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">

</xml_diff>

<commit_message>
RC1.1: ISO7721 pinout fix, CP2102N VBUS divider/RSTb pull-up/VDD bypass, datasheets read locally
- ISO7721 symbol corrected to the TI D/DWV table (2 OUTA, 3 INB, 6 OUTB, 7 INA); UART nets reassigned and re-routed
- CP2102N: VBUS 22.1k/47.5k divider (R38/R39), 1k RSTb pull-up (R40), VDD bypass 4.7uF (C22) per the datasheet
- ISO7721, CP2102N, SRN6045TA datasheets committed as evidence and marked VERIFIED_LOCAL; SRN6045TA-100M inductor closed
- isolation check script/report (3.0 mm in the ISO7721 area, 0.25 mm elsewhere); docs corrected (netclass clearances)
- board re-placed and re-routed: ERC 0, DRC 0 electrical (3 silkscreen warnings), netlist 0 mismatches

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HV1TCrYnLTcNjmYdFqCPLo
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
+++ b/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
@@ -37,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -83,6 +88,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:R62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1271,7 +1279,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>10 uH shielded inductor 6x6 mm (value/Isat per LMR14006 design equations; UNVERIFIED)</t>
+          <t>10 uH shielded inductor 6x6 mm (10 uH +/-20 %, DCR 52 mohm, Irms 3.2 A, Isat 4.6 A: Bourns datasheet read locally)</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1294,9 +1302,9 @@
           <t>Inductor_SMD:L_Bourns_SRN6045TA</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>VERIFIED_LOCAL</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1766,11 +1774,11 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>C7, C15, C20</t>
+          <t>C7, C15, C20, C22</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
@@ -1842,7 +1850,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R17" s="3" t="inlineStr"/>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>CP2102N VDD: 4.7 uF + 0.1 uF required per power pin (Silicon Labs datasheet, read locally)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1938,11 +1950,11 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>R5, R7, R20, R32</t>
+          <t>R5, R7, R20, R32, R40</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
@@ -2014,7 +2026,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R19" s="3" t="inlineStr"/>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>CP2102N RSTb 1 kOhm pull-up to VDD (Silicon Labs datasheet 2.1, read locally)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -2190,11 +2206,11 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>C16, C22</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
@@ -3078,9 +3094,9 @@
           <t>Package_DFN_QFN:SiliconLabs_QFN-20-1EP_3x3mm_P0.5mm_EP1.8x1.8mm</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>VERIFIED_LOCAL</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -3126,7 +3142,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>U7</t>
+          <t>R38</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -3134,32 +3150,32 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>ISO7721</t>
+          <t>22.1k</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>ISO7721 dual-channel digital isolator 1 fwd / 1 rev SOIC-8 (no isolated power)</t>
+          <t>22.1k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>ISO7721DR</t>
+          <t>CRCW060322K1FKEA</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>SOIC-8</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
@@ -3189,7 +3205,7 @@
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>ISO7721DWR (wide body) (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
@@ -3202,7 +3218,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R33" s="3" t="inlineStr"/>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>CP2102N VBUS sense divider (Silicon Labs reference, relayed): 22.1 k upper</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -3210,7 +3230,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>R39</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
@@ -3218,32 +3238,32 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>SHUNT_KELVIN</t>
+          <t>47.5k</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>KK 254 3-pos vertical header (mate 22-01-3037 + 08-50-0114)</t>
+          <t>47.5k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>22-27-2031</t>
+          <t>CRCW060347K5FKEA</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>Molex_KK-254_AE-6410-03A_1x03_P2.54mm_Vertical</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Connector_Molex:Molex_KK-254_AE-6410-03A_1x03_P2.54mm_Vertical</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
@@ -3273,7 +3293,7 @@
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>Molex 22-23-2031 (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
@@ -3288,7 +3308,7 @@
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t>1 IN+, 2 IN-, 3 cable shield (shield joined to GND at this end only)</t>
+          <t>CP2102N VBUS sense divider: 47.5 k lower</t>
         </is>
       </c>
     </row>
@@ -3298,45 +3318,45 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>D5, D6, D7</t>
+          <t>U7</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>1.5SMBJ48A</t>
+          <t>ISO7721</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Unidirectional TVS 48 V standoff 1500 W (K = pin 1)</t>
+          <t>ISO7721 dual-channel digital isolator 1 fwd / 1 rev SOIC-8 (no isolated power)</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>1.5SMBJ48A</t>
+          <t>ISO7721DR</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>SOIC-8</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Diode_SMD:D_SMB</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>VERIFIED_LOCAL</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -3361,12 +3381,12 @@
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Littelfuse 1.5SMC / SMBJ48A (UNVERIFIED alternate)</t>
+          <t>ISO7721DWR (wide body) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 2; 3 needed) or PCBWay source</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
@@ -3374,7 +3394,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R35" s="3" t="inlineStr"/>
+      <c r="R35" s="3" t="inlineStr">
+        <is>
+          <t>Channel A (INA pin 7, host side) -&gt; OUTA pin 2 (MCU RX); channel B (INB pin 3 &lt;- MCU TX) -&gt; OUTB pin 6 (CP2102N RXD)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -3382,40 +3406,40 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>R11, R12, R13</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>SHUNT_KELVIN</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>10 1 % thick film 0603</t>
+          <t>KK 254 3-pos vertical header (mate 22-01-3037 + 08-50-0114)</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>CRCW060310R0FKEA</t>
+          <t>22-27-2031</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>Molex_KK-254_AE-6410-03A_1x03_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Connector_Molex:Molex_KK-254_AE-6410-03A_1x03_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -3445,7 +3469,7 @@
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Molex 22-23-2031 (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr">
@@ -3458,7 +3482,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R36" s="3" t="inlineStr"/>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>1 IN+, 2 IN-, 3 cable shield (shield joined to GND at this end only)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -3466,45 +3494,45 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>C26, C28</t>
+          <t>D5, D6, D7</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>100nF 50V</t>
+          <t>1.5SMBJ48A</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>100 nF 50 V X7R 0603</t>
+          <t>Unidirectional TVS 48 V standoff 1500 W (K = pin 1)</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>GRM188R71H104KA93D</t>
+          <t>1.5SMBJ48A</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Diode_SMD:D_SMB</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -3529,12 +3557,12 @@
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL10B104KB8NNNC (UNVERIFIED alternate)</t>
+          <t>Littelfuse 1.5SMC / SMBJ48A (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P37" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 2; 3 needed) or PCBWay source</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr">
@@ -3542,11 +3570,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R37" s="3" t="inlineStr">
-        <is>
-          <t>Differential filter fc ~80 kHz</t>
-        </is>
-      </c>
+      <c r="R37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -3554,50 +3578,50 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>R11, R12, R13</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>INA228</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>INA228 85 V 20-bit I2C power monitor VSSOP-10 (PIN MAP UNVERIFIED)</t>
+          <t>10 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>INA228AIDGSR</t>
+          <t>CRCW060310R0FKEA</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Package_SO:MSOP-10_3x3mm_P0.5mm</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE (user-confirmed)</t>
+          <t>UNKNOWN (not checked)</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
@@ -3617,7 +3641,7 @@
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>INA228AIDGST (small reel) (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P38" s="3" t="inlineStr">
@@ -3638,30 +3662,30 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>R14, R15, R35, R36</t>
+          <t>C26, C28</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>100nF 50V</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>4.7k 1 % thick film 0603</t>
+          <t>100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>CRCW06034K70FKEA</t>
+          <t>GRM188R71H104KA93D</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -3671,7 +3695,7 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
@@ -3701,7 +3725,7 @@
       </c>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Samsung CL10B104KB8NNNC (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P39" s="3" t="inlineStr">
@@ -3716,7 +3740,7 @@
       </c>
       <c r="R39" s="3" t="inlineStr">
         <is>
-          <t>Fitted; 2.2k alternative for long cables</t>
+          <t>Differential filter fc ~80 kHz</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3750,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
@@ -3734,42 +3758,42 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>PACK_SENSE</t>
+          <t>INA228</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>KK 254 4-pos vertical header (mate 22-01-3047 + 08-50-0114)</t>
+          <t>INA228 85 V 20-bit I2C power monitor VSSOP-10 (PIN MAP UNVERIFIED)</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>22-27-2041</t>
+          <t>INA228AIDGSR</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Connector_Molex:Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Package_SO:MSOP-10_3x3mm_P0.5mm</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>UNKNOWN (not checked)</t>
+          <t>ACTIVE (user-confirmed)</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
@@ -3789,7 +3813,7 @@
       </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>Molex 22-23-2041 (UNVERIFIED alternate)</t>
+          <t>INA228AIDGST (small reel) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P40" s="3" t="inlineStr">
@@ -3802,11 +3826,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R40" s="3" t="inlineStr">
-        <is>
-          <t>1 PACK_INA (upstream of K1), 2 PACK_ADC (separate lead), 3 RELAY_OUT (K1 load side), 4 GND_SENSE = the single logic-GND / pack-negative bond</t>
-        </is>
-      </c>
+      <c r="R40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -3814,20 +3834,20 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>R17, R18</t>
+          <t>R14, R15, R35, R36</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>75k 0.1%</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>75k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
+          <t>4.7k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3837,22 +3857,22 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>TNPW080575K0BEEA</t>
+          <t>CRCW06034K70FKEA</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
@@ -3877,7 +3897,7 @@
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>Susumu RG2012P-series 0.1 %/25 ppm (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P41" s="3" t="inlineStr">
@@ -3890,7 +3910,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R41" s="3" t="inlineStr"/>
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t>Fitted; 2.2k alternative for long cables</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -3898,7 +3922,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -3906,37 +3930,37 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>10k 0.1%</t>
+          <t>PACK_SENSE</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>10k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
+          <t>KK 254 4-pos vertical header (mate 22-01-3047 + 08-50-0114)</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>TNPW080510K0BEEA</t>
+          <t>22-27-2041</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Connector_Molex:Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -3961,7 +3985,7 @@
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Susumu RG2012P-series 0.1 %/25 ppm (UNVERIFIED alternate)</t>
+          <t>Molex 22-23-2041 (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P42" s="3" t="inlineStr">
@@ -3974,7 +3998,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R42" s="3" t="inlineStr"/>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>1 PACK_INA (upstream of K1), 2 PACK_ADC (separate lead), 3 RELAY_OUT (K1 load side), 4 GND_SENSE = the single logic-GND / pack-negative bond</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -3982,45 +4010,45 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>D8, D13, D14</t>
+          <t>R17, R18</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>BAT54S</t>
+          <t>75k 0.1%</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Dual series Schottky SOT-23 (clamp)</t>
+          <t>75k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>BAT54S,215</t>
+          <t>TNPW080575K0BEEA</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_SMD:SOT-23</t>
-        </is>
-      </c>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -4045,7 +4073,7 @@
       </c>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>onsemi BAT54SLT1G (UNVERIFIED alternate)</t>
+          <t>Susumu RG2012P-series 0.1 %/25 ppm (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P43" s="3" t="inlineStr">
@@ -4058,11 +4086,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R43" s="3" t="inlineStr">
-        <is>
-          <t>ARM_SENSE clamp: source impedance 73 k -&gt; back-feed &lt; 60 uA; Blocks VCLAMP -&gt; 3V3: PACK+ back-feed through D8 cannot reach the MCU rail; Lower clamp to GND; upper clamp to the ISOLATED rail VCLAMP (not 3V3)</t>
-        </is>
-      </c>
+      <c r="R43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -4070,7 +4094,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
@@ -4078,32 +4102,32 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ESTOP</t>
+          <t>10k 0.1%</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
+          <t>10k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>Adam Tech</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C</t>
+          <t>TNPW080510K0BEEA</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -4133,12 +4157,12 @@
       </c>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>Phoenix MKDS 1/2-5,08 (different footprint) (UNVERIFIED alternate)</t>
+          <t>Susumu RG2012P-series 0.1 %/25 ppm (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P44" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 5) or PCBWay source</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="Q44" s="3" t="inlineStr">
@@ -4146,11 +4170,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R44" s="3" t="inlineStr">
-        <is>
-          <t>Eaton M22-PV-K02 NC contact in series: pin 1 +12 V, pin 2 post-E-stop node</t>
-        </is>
-      </c>
+      <c r="R44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -4158,45 +4178,45 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>D8, D13, D14</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>BAT54S</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
+          <t>Dual series Schottky SOT-23 (clamp)</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Adam Tech</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C</t>
+          <t>BAT54S,215</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Package_TO_SOT_SMD:SOT-23</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -4221,12 +4241,12 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>Phoenix MKDS 1/2-5,08 (different footprint) (UNVERIFIED alternate)</t>
+          <t>onsemi BAT54SLT1G (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 5) or PCBWay source</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="Q45" s="3" t="inlineStr">
@@ -4236,7 +4256,7 @@
       </c>
       <c r="R45" s="3" t="inlineStr">
         <is>
-          <t>C&amp;K T102SHZQE ARM switch in series</t>
+          <t>ARM_SENSE clamp: source impedance 73 k -&gt; back-feed &lt; 60 uA; Blocks VCLAMP -&gt; 3V3: PACK+ back-feed through D8 cannot reach the MCU rail; Lower clamp to GND; upper clamp to the ISOLATED rail VCLAMP (not 3V3)</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4266,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
@@ -4254,7 +4274,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>K1_COIL</t>
+          <t>ESTOP</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
@@ -4324,7 +4344,7 @@
       </c>
       <c r="R46" s="3" t="inlineStr">
         <is>
-          <t>Durakool DG57CM-5021-76-1012-R coil (12 V). Pin 1 +12 V side, pin 2 MOSFET drain</t>
+          <t>Eaton M22-PV-K02 NC contact in series: pin 1 +12 V, pin 2 post-E-stop node</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4354,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -4342,32 +4362,32 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>IRLML0060</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>N-MOSFET 60 V SOT-23 logic-level (relay low side). RDS(on) not specified at 3.3 V: gate-drive check required</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Infineon</t>
+          <t>Adam Tech</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>IRLML0060TRPBF</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_SMD:SOT-23</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -4397,12 +4417,12 @@
       </c>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>Diodes DMN6140L-7 / AOS AO3400A (30 V) (UNVERIFIED alternate)</t>
+          <t>Phoenix MKDS 1/2-5,08 (different footprint) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P47" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 5) or PCBWay source</t>
         </is>
       </c>
       <c r="Q47" s="3" t="inlineStr">
@@ -4410,7 +4430,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R47" s="3" t="inlineStr"/>
+      <c r="R47" s="3" t="inlineStr">
+        <is>
+          <t>C&amp;K T102SHZQE ARM switch in series</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -4418,7 +4442,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
@@ -4426,37 +4450,37 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>K1_COIL</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>220 1 % thick film 0603</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Adam Tech</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>CRCW0603220RFKEA</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="J48" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
@@ -4481,12 +4505,12 @@
       </c>
       <c r="O48" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Phoenix MKDS 1/2-5,08 (different footprint) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P48" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 5) or PCBWay source</t>
         </is>
       </c>
       <c r="Q48" s="3" t="inlineStr">
@@ -4494,7 +4518,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R48" s="3" t="inlineStr"/>
+      <c r="R48" s="3" t="inlineStr">
+        <is>
+          <t>Durakool DG57CM-5021-76-1012-R coil (12 V). Pin 1 +12 V side, pin 2 MOSFET drain</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -4502,7 +4530,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -4510,37 +4538,37 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>S1M</t>
+          <t>IRLML0060</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>1 A 1000 V rectifier SMA (relay-coil flyback)</t>
+          <t>N-MOSFET 60 V SOT-23 logic-level (relay low side). RDS(on) not specified at 3.3 V: gate-drive check required</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Infineon</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>S1M-13-F</t>
+          <t>IRLML0060TRPBF</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>SMA</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Diode_SMD:D_SMA</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Package_TO_SOT_SMD:SOT-23</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
@@ -4565,7 +4593,7 @@
       </c>
       <c r="O49" s="3" t="inlineStr">
         <is>
-          <t>onsemi/owned 1N5408G (THT) (UNVERIFIED alternate)</t>
+          <t>Diodes DMN6140L-7 / AOS AO3400A (30 V) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P49" s="3" t="inlineStr">
@@ -4578,11 +4606,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R49" s="3" t="inlineStr">
-        <is>
-          <t>Flyback: cathode on +12 V side</t>
-        </is>
-      </c>
+      <c r="R49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -4590,7 +4614,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -4598,12 +4622,12 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>2.2k</t>
+          <t>220</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1 % thick film 0603</t>
+          <t>220 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -4613,7 +4637,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>CRCW06032K20FKEA</t>
+          <t>CRCW0603220RFKEA</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -4674,7 +4698,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -4682,32 +4706,32 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>COIL ON</t>
+          <t>S1M</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>LED amber 0805</t>
+          <t>1 A 1000 V rectifier SMA (relay-coil flyback)</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>150080AS75000</t>
+          <t>S1M-13-F</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>LED_SMD:LED_0805_2012Metric</t>
+          <t>Diode_SMD:D_SMA</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -4737,7 +4761,7 @@
       </c>
       <c r="O51" s="3" t="inlineStr">
         <is>
-          <t>Kingbright APT2012SYC (UNVERIFIED alternate)</t>
+          <t>onsemi/owned 1N5408G (THT) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P51" s="3" t="inlineStr">
@@ -4750,7 +4774,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R51" s="3" t="inlineStr"/>
+      <c r="R51" s="3" t="inlineStr">
+        <is>
+          <t>Flyback: cathode on +12 V side</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -4758,7 +4786,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -4766,12 +4794,12 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>5.6k</t>
+          <t>2.2k</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>5.6k 1 % thick film 0603</t>
+          <t>2.2k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -4781,7 +4809,7 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>CRCW06035K60FKEA</t>
+          <t>CRCW06032K20FKEA</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -4834,11 +4862,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R52" s="3" t="inlineStr">
-        <is>
-          <t>IF &gt;= 1.59 mA at 10.5 V (worst-case VF 1.6 V): 2x saturation margin with CTR_eff = 13 % x 0.8 x 0.8</t>
-        </is>
-      </c>
+      <c r="R52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -4846,45 +4870,45 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>U4, U5</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>VO610A-1</t>
+          <t>COIL ON</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Optocoupler transistor output DIP-4, CTR bin -1 (13 % min @ 1 mA, 40 % min @ 10 mA: user-relayed)</t>
+          <t>LED amber 0805</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>VO610A-1</t>
+          <t>150080AS75000</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>DIP-4</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Package_DIP:DIP-4_W7.62mm</t>
-        </is>
-      </c>
-      <c r="J53" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>LED_SMD:LED_0805_2012Metric</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
@@ -4909,12 +4933,12 @@
       </c>
       <c r="O53" s="3" t="inlineStr">
         <is>
-          <t>Vishay VO610A-2 (63-125 % bin, resistor re-check) (UNVERIFIED alternate)</t>
+          <t>Kingbright APT2012SYC (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P53" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 2) + spares</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="Q53" s="3" t="inlineStr">
@@ -4930,40 +4954,40 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>D11, D12</t>
+          <t>R24</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>5.6k</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Small-signal diode DO-35 (LED reverse clamp)</t>
+          <t>5.6k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>CRCW06035K60FKEA</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>DO-35</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Diode_THT:D_DO-35_SOD27_P7.62mm_Horizontal</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
@@ -4993,12 +5017,12 @@
       </c>
       <c r="O54" s="3" t="inlineStr">
         <is>
-          <t>Vishay 1N4148 (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P54" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 2) or PCBWay source</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="Q54" s="3" t="inlineStr">
@@ -5008,7 +5032,7 @@
       </c>
       <c r="R54" s="3" t="inlineStr">
         <is>
-          <t>Antiparallel across the LED</t>
+          <t>IF &gt;= 1.59 mA at 10.5 V (worst-case VF 1.6 V): 2x saturation margin with CTR_eff = 13 % x 0.8 x 0.8</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5042,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>R25, R29</t>
+          <t>U4, U5</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -5026,37 +5050,37 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>VO610A-1</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>47k 1 % thick film 0603</t>
+          <t>Optocoupler transistor output DIP-4, CTR bin -1 (13 % min @ 1 mA, 40 % min @ 10 mA: user-relayed)</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>CRCW060347K0FKEA</t>
+          <t>VO610A-1</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>DIP-4</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Package_DIP:DIP-4_W7.62mm</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -5081,12 +5105,12 @@
       </c>
       <c r="O55" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Vishay VO610A-2 (63-125 % bin, resistor re-check) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P55" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 2) + spares</t>
         </is>
       </c>
       <c r="Q55" s="3" t="inlineStr">
@@ -5102,7 +5126,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>C30, C31</t>
+          <t>D11, D12</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -5110,32 +5134,32 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>1N4148</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>10 nF 50 V X7R 0603</t>
+          <t>Small-signal diode DO-35 (LED reverse clamp)</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>onsemi</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>GRM188R71H103KA01D</t>
+          <t>1N4148</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>DO-35</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0603_1608Metric</t>
+          <t>Diode_THT:D_DO-35_SOD27_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
@@ -5165,12 +5189,12 @@
       </c>
       <c r="O56" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL10B103KB8NNNC (UNVERIFIED alternate)</t>
+          <t>Vishay 1N4148 (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P56" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 2) or PCBWay source</t>
         </is>
       </c>
       <c r="Q56" s="3" t="inlineStr">
@@ -5178,7 +5202,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R56" s="3" t="inlineStr"/>
+      <c r="R56" s="3" t="inlineStr">
+        <is>
+          <t>Antiparallel across the LED</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -5186,20 +5214,20 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>R26, R27, R28</t>
+          <t>R25, R29</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>4.7k 1 % thick film 1206 (pulse-rated relay-feedback chain)</t>
+          <t>47k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -5209,17 +5237,17 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>CRCW12064K70FKEA</t>
+          <t>CRCW060347K0FKEA</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -5249,7 +5277,7 @@
       </c>
       <c r="O57" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC1206-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P57" s="3" t="inlineStr">
@@ -5270,30 +5298,30 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>C30, C31</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>270k</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>270k 1 % thick film 0603</t>
+          <t>10 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>CRCW0603270KFKEA</t>
+          <t>GRM188R71H103KA01D</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
@@ -5303,7 +5331,7 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -5333,7 +5361,7 @@
       </c>
       <c r="O58" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Samsung CL10B103KB8NNNC (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P58" s="3" t="inlineStr">
@@ -5354,40 +5382,40 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>J7</t>
+          <t>R26, R27, R28</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>TEMP_PROBE</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>PH 2.0 mm 4-pos vertical header (mate PHR-4 + SPH-002T-P0.5S)</t>
+          <t>4.7k 1 % thick film 1206 (pulse-rated relay-feedback chain)</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>B4B-PH-K-S</t>
+          <t>CRCW12064K70FKEA</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Connector_JST:JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+          <t>Resistor_SMD:R_1206_3216Metric</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -5417,7 +5445,7 @@
       </c>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>JST B4B-PH-K-S(LF)(SN) (UNVERIFIED alternate)</t>
+          <t>Yageo RC1206-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="P59" s="3" t="inlineStr">
@@ -5430,11 +5458,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>1 3V3, 2 SDA2, 3 SCL2, 4 GND</t>
-        </is>
-      </c>
+      <c r="R59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -5442,83 +5466,255 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>270k</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>270k 1 % thick film 0603</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Vishay Dale</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>CRCW0603270KFKEA</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>0603</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN (not checked)</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>Mouser / Digi-Key (authorized) - NOT QUERIED</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>NOT CHECKED (distributor sites unreachable from the build environment)</t>
+        </is>
+      </c>
+      <c r="N60" s="3" t="inlineStr">
+        <is>
+          <t>NOT CHECKED</t>
+        </is>
+      </c>
+      <c r="O60" s="3" t="inlineStr">
+        <is>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+        </is>
+      </c>
+      <c r="P60" s="3" t="inlineStr">
+        <is>
+          <t>PCBWay source</t>
+        </is>
+      </c>
+      <c r="Q60" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>J7</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>TEMP_PROBE</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>PH 2.0 mm 4-pos vertical header (mate PHR-4 + SPH-002T-P0.5S)</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>B4B-PH-K-S</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Connector_JST:JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN (not checked)</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>Mouser / Digi-Key (authorized) - NOT QUERIED</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>NOT CHECKED (distributor sites unreachable from the build environment)</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="inlineStr">
+        <is>
+          <t>NOT CHECKED</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>JST B4B-PH-K-S(LF)(SN) (UNVERIFIED alternate)</t>
+        </is>
+      </c>
+      <c r="P61" s="3" t="inlineStr">
+        <is>
+          <t>PCBWay source</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>1 3V3, 2 SDA2, 3 SCL2, 4 GND</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
           <t>R33, R34</t>
         </is>
       </c>
-      <c r="C60" s="3" t="n">
+      <c r="C62" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>100 1 % thick film 0603</t>
         </is>
       </c>
-      <c r="F60" s="3" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>Vishay Dale</t>
         </is>
       </c>
-      <c r="G60" s="3" t="inlineStr">
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>CRCW0603100RFKEA</t>
         </is>
       </c>
-      <c r="H60" s="3" t="inlineStr">
+      <c r="H62" s="3" t="inlineStr">
         <is>
           <t>0603</t>
         </is>
       </c>
-      <c r="I60" s="3" t="inlineStr">
+      <c r="I62" s="3" t="inlineStr">
         <is>
           <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
-      <c r="J60" s="5" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="K60" s="3" t="inlineStr">
+      <c r="K62" s="3" t="inlineStr">
         <is>
           <t>UNKNOWN (not checked)</t>
         </is>
       </c>
-      <c r="L60" s="3" t="inlineStr">
+      <c r="L62" s="3" t="inlineStr">
         <is>
           <t>Mouser / Digi-Key (authorized) - NOT QUERIED</t>
         </is>
       </c>
-      <c r="M60" s="3" t="inlineStr">
+      <c r="M62" s="3" t="inlineStr">
         <is>
           <t>NOT CHECKED (distributor sites unreachable from the build environment)</t>
         </is>
       </c>
-      <c r="N60" s="3" t="inlineStr">
+      <c r="N62" s="3" t="inlineStr">
         <is>
           <t>NOT CHECKED</t>
         </is>
       </c>
-      <c r="O60" s="3" t="inlineStr">
+      <c r="O62" s="3" t="inlineStr">
         <is>
           <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
-      <c r="P60" s="3" t="inlineStr">
+      <c r="P62" s="3" t="inlineStr">
         <is>
           <t>PCBWay source</t>
         </is>
       </c>
-      <c r="Q60" s="3" t="inlineStr">
+      <c r="Q62" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="R60" s="3" t="inlineStr"/>
+      <c r="R62" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
RC1.2: CP2102N VBUS divider margin (R38 19.1k), protection marked not fully closed, isolation-rule activity check
- R38 22.1k -> 19.1k from the CP2102N datasheet limits (VIH = VDD-0.6 V; +0.12 V at VBUS 4.40 V / VDD 3.6 V / 1 %); value change only, layout unchanged
- pack-sense protection: model PASS but not closed (ERJ-P08F pulse rating, 1.5SMBJ48A leakage unread); surge-capability numbers labelled model results
- ISOLATION_RULE_CHECK: the .kicad_dru is applied from a fresh folder; pack-net rule documented as a low-voltage sense-net rule
- connector drawings still not available: footprints unchanged, item open
- ERC 0, DRC 0, unconnected 0, netlist 0 mismatches, polarity none; no Gerbers in the package

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HV1TCrYnLTcNjmYdFqCPLo
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
+++ b/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
@@ -3405,12 +3405,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>22.1k</t>
+          <t>19.1k</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>22.1k 1 % thick film 0603</t>
+          <t>19.1k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>CRCW060322K1FKEA</t>
+          <t>CRCW060319K1FKEA</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="T33" s="3" t="inlineStr">
         <is>
-          <t>CP2102N VBUS sense divider (Silicon Labs reference, relayed): 22.1 k upper</t>
+          <t>CP2102N VBUS sense divider upper resistor: Silicon Labs reference uses 22.1 k; 19.1 k gives positive margin to VIH = VDD-0.6 V at VBUS 4.40 V / VDD 3.6 V / 1 % resistors (see calculations 8)</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>CP2102N VBUS sense divider: 47.5 k lower</t>
+          <t>CP2102N VBUS sense divider lower resistor (Silicon Labs reference value)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RC1.2d: Panasonic ERJ-P08 catalog and Samtec FTSH catalog page recorded; Molex pages repeated (no drawing)
- ERJ-P08F47R0V / ERJ-P08F10R0V: part-number scheme, 0.66 W, 500 V limiting / 1000 V overload, ESD 3 kV/150 pF read locally; no us-ms pulse curve published
- protection: PASS for the defined transient on datasheet-verified limits; TVS leakage vs temperature and resistor thermal-pulse curve remain first-article items
- Samtec FTSH-105-01-L-DV-K part number/pitch/tail span confirmed; land pattern and key position still open; Molex sales drawings (*_sd.pdf) still needed
- no board change: ERC 0, DRC 0, unconnected 0, netlist 0 mismatches, polarity none, isolation >= 1.0 mm

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HV1TCrYnLTcNjmYdFqCPLo
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
+++ b/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
@@ -2777,7 +2777,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+          <t>confirmed (Samtec FTSH catalog part-number decode, read locally)</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -3809,7 +3809,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+          <t>matches the Panasonic part-number scheme (catalog read locally); distributor listing not checked</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+          <t>confirmed (Bourns datasheet table, read locally)</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+          <t>matches the Panasonic part-number scheme (catalog read locally); distributor listing not checked</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">

</xml_diff>

<commit_message>
RC1.2e: Samtec J9 land pattern (0.74x2.79, rev H), D15 differential clamp across INA228 IN+/IN-, protection and connector audit; ERJ-P08 pulse capability re-opened
- J9 generic footprint replaced by OSBAMS_Rev2:FTSH-105-01-L-DV-K from the Samtec recommended layout rev H; breakout re-routed
- D15 SMF12CA bidirectional TVS across INA_INP/INA_INN (INA228 differential limit +/-40 V; one Kelvin lead open)
- CONTROLLER_PROTECTION_AND_CONNECTOR_AUDIT.md (PASS / CHANGE REQUIRED / FIRST-ARTICLE VALIDATION / REMAINING FABRICATION BLOCKERS)
- rs_pulse_rating back to UNVERIFIED/critical; Molex J5/J6 stay open (3D drawing without dimensions); evidence PDFs committed
- ERC 0, DRC 0, unconnected 0, netlist 0 mismatches (405 pads), polarity OK, isolation >= 1.0 mm; 181 tests pass

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HV1TCrYnLTcNjmYdFqCPLo
</commit_message>
<xml_diff>
--- a/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
+++ b/Hardware/Rev2_Controller/OSBAMS_Rev2_RELEASE_CANDIDATE_1/OSBAMS_Rev2_RC1_BOM.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T64"/>
+  <dimension ref="A1:T65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -486,7 +486,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RC1.2 - REVIEW CANDIDATE - NOT RELEASED FOR FABRICATION</t>
+          <t>RC1.2e - REVIEW CANDIDATE - NOT RELEASED FOR FABRICATION</t>
         </is>
       </c>
     </row>
@@ -2782,12 +2782,12 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>PinHeader_2x05_P1.27mm_Vertical_SMD</t>
+          <t>FTSH-105-01-L-DV-K</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Connector_PinHeader_1.27mm:PinHeader_2x05_P1.27mm_Vertical_SMD</t>
+          <t>OSBAMS_Rev2:FTSH-105-01-L-DV-K</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
@@ -4058,33 +4058,33 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>C26, C28</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>100nF 50V</t>
+          <t>SMF12CA</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>100 nF 50 V X7R 0603</t>
+          <t>Bidirectional TVS 12 V standoff 200 W SMF (differential clamp IN+/IN-)</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Littelfuse</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>GRM188R71H104KA93D</t>
+          <t>SMF12CA</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -4094,12 +4094,12 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>D_SMF</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0603_1608Metric</t>
+          <t>Diode_SMD:D_SMF</t>
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
@@ -4129,12 +4129,12 @@
       </c>
       <c r="Q40" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL10B104KB8NNNC (UNVERIFIED alternate)</t>
+          <t>Bourns SMF12CA / Vishay SMF12A (bidirectional) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R40" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>PCBWay source (datasheet NOT yet read)</t>
         </is>
       </c>
       <c r="S40" s="3" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>Differential filter fc ~80 kHz</t>
+          <t>Differential clamp across the INA228 IN+/IN- pins (one-Kelvin-lead-open / late-connect: INA228 differential abs max is +/-40 V). Bidirectional, VRWM 12 V &gt;&gt; 50 mV full-scale shunt signal</t>
         </is>
       </c>
     </row>
@@ -4154,33 +4154,33 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>C26, C28</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>INA228</t>
+          <t>100nF 50V</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>INA228 85 V 20-bit I2C power monitor VSSOP-10 (PIN MAP UNVERIFIED)</t>
+          <t>100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>INA228AIDGSR</t>
+          <t>GRM188R71H104KA93D</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -4190,22 +4190,22 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>MSOP-10</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Package_SO:MSOP-10_3x3mm_P0.5mm</t>
-        </is>
-      </c>
-      <c r="L41" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE (user-confirmed)</t>
+          <t>UNKNOWN (not checked)</t>
         </is>
       </c>
       <c r="N41" s="3" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="Q41" s="3" t="inlineStr">
         <is>
-          <t>INA228AIDGST (small reel) (UNVERIFIED alternate)</t>
+          <t>Samsung CL10B104KB8NNNC (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R41" s="3" t="inlineStr">
@@ -4238,7 +4238,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T41" s="3" t="inlineStr"/>
+      <c r="T41" s="3" t="inlineStr">
+        <is>
+          <t>Differential filter fc ~80 kHz</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -4246,7 +4250,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>R41</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
@@ -4257,47 +4261,47 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>INA228</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>47 ohm 1 % 1206 anti-surge (pulse-withstanding) thick film: pack-sense surge limiting</t>
+          <t>INA228 85 V 20-bit I2C power monitor VSSOP-10 (PIN MAP UNVERIFIED)</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>ERJ-P08F47R0V</t>
+          <t>INA228AIDGSR</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>matches the Panasonic part-number scheme (catalog read locally); distributor listing not checked</t>
+          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>MSOP-10</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
-        </is>
-      </c>
-      <c r="L42" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Package_SO:MSOP-10_3x3mm_P0.5mm</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>UNKNOWN (not checked)</t>
+          <t>ACTIVE (user-confirmed)</t>
         </is>
       </c>
       <c r="N42" s="3" t="inlineStr">
@@ -4317,12 +4321,12 @@
       </c>
       <c r="Q42" s="3" t="inlineStr">
         <is>
-          <t>Vishay CRCW1206 pulse-rated series / Bourns CR1206-FX-pulse series (pulse rating to be confirmed) (UNVERIFIED alternate)</t>
+          <t>INA228AIDGST (small reel) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R42" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source (orderable suffix to be confirmed)</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="S42" s="3" t="inlineStr">
@@ -4330,11 +4334,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T42" s="3" t="inlineStr">
-        <is>
-          <t>Surge-limiting series resistor UPSTREAM of D7 (Rev.1.2): VBUS input draws ~50 uA so the DC error is negligible</t>
-        </is>
-      </c>
+      <c r="T42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -4342,48 +4342,48 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>R14, R15, R35, R36</t>
+          <t>R41</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>47</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>4.7k 1 % thick film 0603</t>
+          <t>47 ohm 1 % 1206 anti-surge (pulse-withstanding) thick film: pack-sense surge limiting</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>CRCW06034K70FKEA</t>
+          <t>ERJ-P08F47R0V</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+          <t>matches the Panasonic part-number scheme (catalog read locally); distributor listing not checked</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Resistor_SMD:R_1206_3216Metric</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
@@ -4413,12 +4413,12 @@
       </c>
       <c r="Q43" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Vishay CRCW1206 pulse-rated series / Bourns CR1206-FX-pulse series (pulse rating to be confirmed) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R43" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>PCBWay source (orderable suffix to be confirmed)</t>
         </is>
       </c>
       <c r="S43" s="3" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="T43" s="3" t="inlineStr">
         <is>
-          <t>Fitted; 2.2k alternative for long cables</t>
+          <t>Surge-limiting series resistor UPSTREAM of D7 (Rev.1.2): VBUS input draws ~50 uA so the DC error is negligible</t>
         </is>
       </c>
     </row>
@@ -4438,33 +4438,33 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>R14, R15, R35, R36</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>PACK_SENSE</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>KK 254 4-pos vertical header (mate 22-01-3047 + 08-50-0114)</t>
+          <t>4.7k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>22-27-2041</t>
+          <t>CRCW06034K70FKEA</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -4474,12 +4474,12 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Connector_Molex:Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="Q44" s="3" t="inlineStr">
         <is>
-          <t>Molex 22-23-2041 (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R44" s="3" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>1 PACK_INA (upstream of K1), 2 PACK_ADC (separate lead), 3 RELAY_OUT (K1 load side), 4 GND_SENSE = the single logic-GND / pack-negative bond</t>
+          <t>Fitted; 2.2k alternative for long cables</t>
         </is>
       </c>
     </row>
@@ -4534,33 +4534,33 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>R17, R18</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>75k 0.1%</t>
+          <t>PACK_SENSE</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>75k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
+          <t>KK 254 4-pos vertical header (mate 22-01-3047 + 08-50-0114)</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>TNPW080575K0BEEA</t>
+          <t>22-27-2041</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -4570,17 +4570,17 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0805_2012Metric</t>
-        </is>
-      </c>
-      <c r="L45" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Connector_Molex:Molex_KK-254_AE-6410-04A_1x04_P2.54mm_Vertical</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="Q45" s="3" t="inlineStr">
         <is>
-          <t>Susumu RG2012P-series 0.1 %/25 ppm (UNVERIFIED alternate)</t>
+          <t>Molex 22-23-2041 (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R45" s="3" t="inlineStr">
@@ -4618,7 +4618,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T45" s="3" t="inlineStr"/>
+      <c r="T45" s="3" t="inlineStr">
+        <is>
+          <t>1 PACK_INA (upstream of K1), 2 PACK_ADC (separate lead), 3 RELAY_OUT (K1 load side), 4 GND_SENSE = the single logic-GND / pack-negative bond</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -4626,23 +4630,23 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R17, R18</t>
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>10k 0.1%</t>
+          <t>75k 0.1%</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>10k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
+          <t>75k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -4652,7 +4656,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>TNPW080510K0BEEA</t>
+          <t>TNPW080575K0BEEA</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -4718,33 +4722,33 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>D8, D13, D14</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>BAT54S</t>
+          <t>10k 0.1%</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Dual series Schottky SOT-23 (clamp)</t>
+          <t>10k 0.1 % 25 ppm thin film 0805 (ADC divider)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>BAT54S,215</t>
+          <t>TNPW080510K0BEEA</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -4754,17 +4758,17 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_SMD:SOT-23</t>
-        </is>
-      </c>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Resistor_SMD:R_0805_2012Metric</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr">
@@ -4789,7 +4793,7 @@
       </c>
       <c r="Q47" s="3" t="inlineStr">
         <is>
-          <t>onsemi BAT54SLT1G (UNVERIFIED alternate)</t>
+          <t>Susumu RG2012P-series 0.1 %/25 ppm (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R47" s="3" t="inlineStr">
@@ -4802,11 +4806,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T47" s="3" t="inlineStr">
-        <is>
-          <t>ARM_SENSE clamp: source impedance 73 k -&gt; back-feed &lt; 60 uA; Blocks VCLAMP -&gt; 3V3: PACK+ back-feed through D8 cannot reach the MCU rail; Lower clamp to GND; upper clamp to the ISOLATED rail VCLAMP (not 3V3)</t>
-        </is>
-      </c>
+      <c r="T47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -4814,53 +4814,53 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>D8, D13, D14</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>ESTOP</t>
+          <t>BAT54S</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
+          <t>Dual series Schottky SOT-23 (clamp)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Adam Tech</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C</t>
+          <t>BAT54S,215</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>confirmed (Adam Tech drawing EB21A-XX-C, read locally; owned part)</t>
+          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>EB21A-02-C</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>OSBAMS_Rev2:EB21A-02-C</t>
-        </is>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Package_TO_SOT_SMD:SOT-23</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr">
@@ -4885,12 +4885,12 @@
       </c>
       <c r="Q48" s="3" t="inlineStr">
         <is>
-          <t>Phoenix MKDS 1/2-5,08 (different footprint) (UNVERIFIED alternate)</t>
+          <t>onsemi BAT54SLT1G (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R48" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 5) or PCBWay source</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="S48" s="3" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="T48" s="3" t="inlineStr">
         <is>
-          <t>Eaton M22-PV-K02 NC contact in series: pin 1 +12 V, pin 2 post-E-stop node</t>
+          <t>ARM_SENSE clamp: source impedance 73 k -&gt; back-feed &lt; 60 uA; Blocks VCLAMP -&gt; 3V3: PACK+ back-feed through D8 cannot reach the MCU rail; Lower clamp to GND; upper clamp to the ISOLATED rail VCLAMP (not 3V3)</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C49" s="3" t="n">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ESTOP</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="T49" s="3" t="inlineStr">
         <is>
-          <t>C&amp;K T102SHZQE ARM switch in series</t>
+          <t>Eaton M22-PV-K02 NC contact in series: pin 1 +12 V, pin 2 post-E-stop node</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5006,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="C50" s="3" t="n">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>K1_COIL</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="T50" s="3" t="inlineStr">
         <is>
-          <t>Durakool DG57CM-5021-76-1012-R coil (12 V). Pin 1 +12 V side, pin 2 MOSFET drain</t>
+          <t>C&amp;K T102SHZQE ARM switch in series</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="C51" s="3" t="n">
@@ -5113,37 +5113,37 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>IRLML0060</t>
+          <t>K1_COIL</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>N-MOSFET 60 V SOT-23 logic-level (relay low side). RDS(on) not specified at 3.3 V: gate-drive check required</t>
+          <t>2-pos 5.00 mm right-angle screw terminal, 8 A / 300 V (footprint from Adam Tech drawing EB21A-XX-C rev B)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>Infineon</t>
+          <t>Adam Tech</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>IRLML0060TRPBF</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+          <t>confirmed (Adam Tech drawing EB21A-XX-C, read locally; owned part)</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>EB21A-02-C</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Package_TO_SOT_SMD:SOT-23</t>
+          <t>OSBAMS_Rev2:EB21A-02-C</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr">
@@ -5173,12 +5173,12 @@
       </c>
       <c r="Q51" s="3" t="inlineStr">
         <is>
-          <t>Diodes DMN6140L-7 / AOS AO3400A (30 V) (UNVERIFIED alternate)</t>
+          <t>Phoenix MKDS 1/2-5,08 (different footprint) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R51" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 5) or PCBWay source</t>
         </is>
       </c>
       <c r="S51" s="3" t="inlineStr">
@@ -5186,7 +5186,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T51" s="3" t="inlineStr"/>
+      <c r="T51" s="3" t="inlineStr">
+        <is>
+          <t>Durakool DG57CM-5021-76-1012-R coil (12 V). Pin 1 +12 V side, pin 2 MOSFET drain</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -5194,7 +5198,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C52" s="3" t="n">
@@ -5205,22 +5209,22 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>IRLML0060</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>220 1 % thick film 0603</t>
+          <t>N-MOSFET 60 V SOT-23 logic-level (relay low side). RDS(on) not specified at 3.3 V: gate-drive check required</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Infineon</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>CRCW0603220RFKEA</t>
+          <t>IRLML0060TRPBF</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -5230,17 +5234,17 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="L52" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Package_TO_SOT_SMD:SOT-23</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr">
@@ -5265,7 +5269,7 @@
       </c>
       <c r="Q52" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Diodes DMN6140L-7 / AOS AO3400A (30 V) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R52" s="3" t="inlineStr">
@@ -5286,7 +5290,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="C53" s="3" t="n">
@@ -5297,22 +5301,22 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>S1M</t>
+          <t>220</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>1 A 1000 V rectifier SMA (relay-coil flyback)</t>
+          <t>220 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>S1M-13-F</t>
+          <t>CRCW0603220RFKEA</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -5322,12 +5326,12 @@
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>SMA</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Diode_SMD:D_SMA</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L53" s="5" t="inlineStr">
@@ -5357,7 +5361,7 @@
       </c>
       <c r="Q53" s="3" t="inlineStr">
         <is>
-          <t>onsemi/owned 1N5408G (THT) (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R53" s="3" t="inlineStr">
@@ -5370,11 +5374,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T53" s="3" t="inlineStr">
-        <is>
-          <t>Flyback: cathode on +12 V side</t>
-        </is>
-      </c>
+      <c r="T53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="C54" s="3" t="n">
@@ -5393,22 +5393,22 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>2.2k</t>
+          <t>S1M</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>2.2k 1 % thick film 0603</t>
+          <t>1 A 1000 V rectifier SMA (relay-coil flyback)</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>CRCW06032K20FKEA</t>
+          <t>S1M-13-F</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -5418,12 +5418,12 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>SMA</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Diode_SMD:D_SMA</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="Q54" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>onsemi/owned 1N5408G (THT) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R54" s="3" t="inlineStr">
@@ -5466,7 +5466,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T54" s="3" t="inlineStr"/>
+      <c r="T54" s="3" t="inlineStr">
+        <is>
+          <t>Flyback: cathode on +12 V side</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -5474,7 +5478,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -5485,22 +5489,22 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>COIL ON</t>
+          <t>2.2k</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>LED amber 0805</t>
+          <t>2.2k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>150080AS75000</t>
+          <t>CRCW06032K20FKEA</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -5510,12 +5514,12 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>LED_SMD:LED_0805_2012Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L55" s="5" t="inlineStr">
@@ -5545,7 +5549,7 @@
       </c>
       <c r="Q55" s="3" t="inlineStr">
         <is>
-          <t>Kingbright APT2012SYC (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R55" s="3" t="inlineStr">
@@ -5566,7 +5570,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
@@ -5577,22 +5581,22 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>5.6k</t>
+          <t>COIL ON</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>5.6k 1 % thick film 0603</t>
+          <t>LED amber 0805</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>CRCW06035K60FKEA</t>
+          <t>150080AS75000</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -5602,12 +5606,12 @@
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>LED_SMD:LED_0805_2012Metric</t>
         </is>
       </c>
       <c r="L56" s="5" t="inlineStr">
@@ -5637,7 +5641,7 @@
       </c>
       <c r="Q56" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Kingbright APT2012SYC (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R56" s="3" t="inlineStr">
@@ -5650,11 +5654,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T56" s="3" t="inlineStr">
-        <is>
-          <t>IF &gt;= 1.59 mA at 10.5 V (worst-case VF 1.6 V): 2x saturation margin with CTR_eff = 13 % x 0.8 x 0.8</t>
-        </is>
-      </c>
+      <c r="T56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -5662,33 +5662,33 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>U4, U5</t>
+          <t>R24</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>VO610A-1</t>
+          <t>5.6k</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Optocoupler transistor output DIP-4, CTR bin -1 (13 % min @ 1 mA, 40 % min @ 10 mA: user-relayed)</t>
+          <t>5.6k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>VO610A-1</t>
+          <t>CRCW06035K60FKEA</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -5698,17 +5698,17 @@
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>DIP-4</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Package_DIP:DIP-4_W7.62mm</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>USER_RELAYED_MANUFACTURER</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="M57" s="3" t="inlineStr">
@@ -5733,12 +5733,12 @@
       </c>
       <c r="Q57" s="3" t="inlineStr">
         <is>
-          <t>Vishay VO610A-2 (63-125 % bin, resistor re-check) (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R57" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 2) + spares</t>
+          <t>PCBWay source</t>
         </is>
       </c>
       <c r="S57" s="3" t="inlineStr">
@@ -5746,7 +5746,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T57" s="3" t="inlineStr"/>
+      <c r="T57" s="3" t="inlineStr">
+        <is>
+          <t>IF &gt;= 1.59 mA at 10.5 V (worst-case VF 1.6 V): 2x saturation margin with CTR_eff = 13 % x 0.8 x 0.8</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -5754,7 +5758,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>D11, D12</t>
+          <t>U4, U5</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -5765,22 +5769,22 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>VO610A-1</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Small-signal diode DO-35 (LED reverse clamp)</t>
+          <t>Optocoupler transistor output DIP-4, CTR bin -1 (13 % min @ 1 mA, 40 % min @ 10 mA: user-relayed)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>VO610A-1</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -5790,17 +5794,17 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>DO-35</t>
+          <t>DIP-4</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Diode_THT:D_DO-35_SOD27_P7.62mm_Horizontal</t>
-        </is>
-      </c>
-      <c r="L58" s="5" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
+          <t>Package_DIP:DIP-4_W7.62mm</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>USER_RELAYED_MANUFACTURER</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr">
@@ -5825,12 +5829,12 @@
       </c>
       <c r="Q58" s="3" t="inlineStr">
         <is>
-          <t>Vishay 1N4148 (UNVERIFIED alternate)</t>
+          <t>Vishay VO610A-2 (63-125 % bin, resistor re-check) (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R58" s="3" t="inlineStr">
         <is>
-          <t>CONSIGN (owned: 2) or PCBWay source</t>
+          <t>CONSIGN (owned: 2) + spares</t>
         </is>
       </c>
       <c r="S58" s="3" t="inlineStr">
@@ -5838,11 +5842,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T58" s="3" t="inlineStr">
-        <is>
-          <t>Antiparallel across the LED</t>
-        </is>
-      </c>
+      <c r="T58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>R25, R29</t>
+          <t>D11, D12</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
@@ -5861,22 +5861,22 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>47k</t>
+          <t>1N4148</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>47k 1 % thick film 0603</t>
+          <t>Small-signal diode DO-35 (LED reverse clamp)</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>onsemi</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>CRCW060347K0FKEA</t>
+          <t>1N4148</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
@@ -5886,12 +5886,12 @@
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>DO-35</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Diode_THT:D_DO-35_SOD27_P7.62mm_Horizontal</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -5921,12 +5921,12 @@
       </c>
       <c r="Q59" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Vishay 1N4148 (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R59" s="3" t="inlineStr">
         <is>
-          <t>PCBWay source</t>
+          <t>CONSIGN (owned: 2) or PCBWay source</t>
         </is>
       </c>
       <c r="S59" s="3" t="inlineStr">
@@ -5934,7 +5934,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T59" s="3" t="inlineStr"/>
+      <c r="T59" s="3" t="inlineStr">
+        <is>
+          <t>Antiparallel across the LED</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -5942,7 +5946,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>C30, C31</t>
+          <t>R25, R29</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
@@ -5953,22 +5957,22 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>10 nF 50 V X7R 0603</t>
+          <t>47k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>GRM188R71H103KA01D</t>
+          <t>CRCW060347K0FKEA</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -5983,7 +5987,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0603_1608Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -6013,7 +6017,7 @@
       </c>
       <c r="Q60" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL10B103KB8NNNC (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R60" s="3" t="inlineStr">
@@ -6034,33 +6038,33 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>R26, R27, R28</t>
+          <t>C30, C31</t>
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>4.7k 1 % thick film 1206 (pulse-rated relay-feedback chain)</t>
+          <t>10 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>CRCW12064K70FKEA</t>
+          <t>GRM188R71H103KA01D</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -6070,12 +6074,12 @@
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_1206_3216Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -6105,7 +6109,7 @@
       </c>
       <c r="Q61" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC1206-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Samsung CL10B103KB8NNNC (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R61" s="3" t="inlineStr">
@@ -6126,23 +6130,23 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R26, R27, R28</t>
         </is>
       </c>
       <c r="C62" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>270k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>270k 1 % thick film 0603</t>
+          <t>4.7k 1 % thick film 1206 (pulse-rated relay-feedback chain)</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -6152,7 +6156,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>CRCW0603270KFKEA</t>
+          <t>CRCW12064K70FKEA</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
@@ -6162,12 +6166,12 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0603_1608Metric</t>
+          <t>Resistor_SMD:R_1206_3216Metric</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
@@ -6197,7 +6201,7 @@
       </c>
       <c r="Q62" s="3" t="inlineStr">
         <is>
-          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
+          <t>Yageo RC1206-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R62" s="3" t="inlineStr">
@@ -6218,7 +6222,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>J7</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="C63" s="3" t="n">
@@ -6229,22 +6233,22 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>TEMP_PROBE</t>
+          <t>270k</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>PH 2.0 mm 4-pos vertical header (mate PHR-4 + SPH-002T-P0.5S)</t>
+          <t>270k 1 % thick film 0603</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>B4B-PH-K-S</t>
+          <t>CRCW0603270KFKEA</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -6254,12 +6258,12 @@
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+          <t>0603</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Connector_JST:JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr">
@@ -6289,7 +6293,7 @@
       </c>
       <c r="Q63" s="3" t="inlineStr">
         <is>
-          <t>JST B4B-PH-K-S(LF)(SN) (UNVERIFIED alternate)</t>
+          <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
       <c r="R63" s="3" t="inlineStr">
@@ -6302,11 +6306,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T63" s="3" t="inlineStr">
-        <is>
-          <t>1 3V3, 2 SDA2, 3 SCL2, 4 GND</t>
-        </is>
-      </c>
+      <c r="T63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -6314,91 +6314,187 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
+          <t>J7</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>TEMP_PROBE</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>PH 2.0 mm 4-pos vertical header (mate PHR-4 + SPH-002T-P0.5S)</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>B4B-PH-K-S</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Connector_JST:JST_PH_B4B-PH-K_1x04_P2.00mm_Vertical</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>UNKNOWN (not checked)</t>
+        </is>
+      </c>
+      <c r="N64" s="3" t="inlineStr">
+        <is>
+          <t>Mouser / Digi-Key (authorized) - NOT QUERIED</t>
+        </is>
+      </c>
+      <c r="O64" s="3" t="inlineStr">
+        <is>
+          <t>NOT CHECKED (distributor sites unreachable from the build environment)</t>
+        </is>
+      </c>
+      <c r="P64" s="3" t="inlineStr">
+        <is>
+          <t>NOT CHECKED</t>
+        </is>
+      </c>
+      <c r="Q64" s="3" t="inlineStr">
+        <is>
+          <t>JST B4B-PH-K-S(LF)(SN) (UNVERIFIED alternate)</t>
+        </is>
+      </c>
+      <c r="R64" s="3" t="inlineStr">
+        <is>
+          <t>PCBWay source</t>
+        </is>
+      </c>
+      <c r="S64" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="T64" s="3" t="inlineStr">
+        <is>
+          <t>1 3V3, 2 SDA2, 3 SCL2, 4 GND</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
           <t>R33, R34</t>
         </is>
       </c>
-      <c r="C64" s="3" t="n">
+      <c r="C65" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D64" s="3" t="n">
+      <c r="D65" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E65" s="3" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>100 1 % thick film 0603</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Vishay Dale</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>CRCW0603100RFKEA</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr">
+      <c r="I65" s="3" t="inlineStr">
         <is>
           <t>orderable suffix NOT yet confirmed against a distributor/manufacturer listing</t>
         </is>
       </c>
-      <c r="J64" s="3" t="inlineStr">
+      <c r="J65" s="3" t="inlineStr">
         <is>
           <t>0603</t>
         </is>
       </c>
-      <c r="K64" s="3" t="inlineStr">
+      <c r="K65" s="3" t="inlineStr">
         <is>
           <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
-      <c r="L64" s="5" t="inlineStr">
+      <c r="L65" s="5" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="M64" s="3" t="inlineStr">
+      <c r="M65" s="3" t="inlineStr">
         <is>
           <t>UNKNOWN (not checked)</t>
         </is>
       </c>
-      <c r="N64" s="3" t="inlineStr">
+      <c r="N65" s="3" t="inlineStr">
         <is>
           <t>Mouser / Digi-Key (authorized) - NOT QUERIED</t>
         </is>
       </c>
-      <c r="O64" s="3" t="inlineStr">
+      <c r="O65" s="3" t="inlineStr">
         <is>
           <t>NOT CHECKED (distributor sites unreachable from the build environment)</t>
         </is>
       </c>
-      <c r="P64" s="3" t="inlineStr">
+      <c r="P65" s="3" t="inlineStr">
         <is>
           <t>NOT CHECKED</t>
         </is>
       </c>
-      <c r="Q64" s="3" t="inlineStr">
+      <c r="Q65" s="3" t="inlineStr">
         <is>
           <t>Yageo RC0603-FR-07 series (UNVERIFIED alternate)</t>
         </is>
       </c>
-      <c r="R64" s="3" t="inlineStr">
+      <c r="R65" s="3" t="inlineStr">
         <is>
           <t>PCBWay source</t>
         </is>
       </c>
-      <c r="S64" s="3" t="inlineStr">
+      <c r="S65" s="3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="T64" s="3" t="inlineStr"/>
+      <c r="T65" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>